<commit_message>
lisskins-steamdt-compare: data rebuild with category/rarity for all 134 items
</commit_message>
<xml_diff>
--- a/lisskins-steamdt-compare/comparison.xlsx
+++ b/lisskins-steamdt-compare/comparison.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
-  <si>
-    <t>Сравнение цен LIS-SKINS vs SteamDT (Steam/BUFF/YouPin), обновлено 18.07.2026 17:42</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="171">
+  <si>
+    <t>Сравнение цен LIS-SKINS vs SteamDT (Steam/BUFF/YouPin), обновлено 18.07.2026 17:57</t>
   </si>
   <si>
     <t>Список: https://lis-skins.com/ru/market/cs2/?user_list_id=01kvbgbzhn0acjzykwfagmc96y</t>
@@ -58,18 +58,42 @@
     <t>Разница %</t>
   </si>
   <si>
+    <t>Категория</t>
+  </si>
+  <si>
+    <t>Редкость</t>
+  </si>
+  <si>
     <t>MP9 | Pandora's Box (Factory New)</t>
   </si>
   <si>
+    <t>SMG</t>
+  </si>
+  <si>
+    <t>Mil-Spec Grade</t>
+  </si>
+  <si>
     <t>MP9 | Stained Glass (Factory New)</t>
   </si>
   <si>
+    <t>Restricted</t>
+  </si>
+  <si>
     <t>USP-S | Whiteout (Minimal Wear)</t>
   </si>
   <si>
+    <t>Pistol</t>
+  </si>
+  <si>
+    <t>Classified</t>
+  </si>
+  <si>
     <t>M4A4 | Desolate Space (Factory New)</t>
   </si>
   <si>
+    <t>Rifle</t>
+  </si>
+  <si>
     <t>AK-47 | Point Disarray (Factory New)</t>
   </si>
   <si>
@@ -79,6 +103,12 @@
     <t>AWP | Containment Breach (Field-Tested)</t>
   </si>
   <si>
+    <t>Sniper Rifle</t>
+  </si>
+  <si>
+    <t>Covert</t>
+  </si>
+  <si>
     <t>MP9 | Dark Age (Factory New)</t>
   </si>
   <si>
@@ -139,6 +169,12 @@
     <t>Chem-Haz Capitaine | Gendarmerie Nationale</t>
   </si>
   <si>
+    <t>Agent</t>
+  </si>
+  <si>
+    <t>Superior</t>
+  </si>
+  <si>
     <t>SG 553 | Integrale (Minimal Wear)</t>
   </si>
   <si>
@@ -151,6 +187,9 @@
     <t>Nova | Sobek's Bite (Factory New)</t>
   </si>
   <si>
+    <t>Shotgun</t>
+  </si>
+  <si>
     <t>M4A4 | Polysoup (Minimal Wear)</t>
   </si>
   <si>
@@ -166,9 +205,18 @@
     <t>Sticker | Movistar Riders (Holo) | Stockholm 2021</t>
   </si>
   <si>
+    <t>Sticker</t>
+  </si>
+  <si>
+    <t>Remarkable</t>
+  </si>
+  <si>
     <t>'The Doctor' Romanov | Sabre</t>
   </si>
   <si>
+    <t>Master</t>
+  </si>
+  <si>
     <t>Five-SeveN | Copper Galaxy (Minimal Wear)</t>
   </si>
   <si>
@@ -178,12 +226,18 @@
     <t>Sticker | Great Wave (Foil)</t>
   </si>
   <si>
+    <t>Exotic</t>
+  </si>
+  <si>
     <t>M4A4 | Evil Daimyo (Factory New)</t>
   </si>
   <si>
     <t>SG 553 | Candy Apple (Factory New)</t>
   </si>
   <si>
+    <t>Industrial Grade</t>
+  </si>
+  <si>
     <t>AWP | Exoskeleton (Minimal Wear)</t>
   </si>
   <si>
@@ -211,9 +265,15 @@
     <t>Osiris | Elite Crew</t>
   </si>
   <si>
+    <t>Exceptional</t>
+  </si>
+  <si>
     <t>B Squadron Officer | SAS</t>
   </si>
   <si>
+    <t>Distinguished</t>
+  </si>
+  <si>
     <t>AUG | Carved Jade (Minimal Wear)</t>
   </si>
   <si>
@@ -226,15 +286,15 @@
     <t>MP7 | Fade (Minimal Wear)</t>
   </si>
   <si>
+    <t>MP7 | Fade (Field-Tested)</t>
+  </si>
+  <si>
+    <t>Sticker | Great Wave (Holo)</t>
+  </si>
+  <si>
     <t>Sticker | 9z Team (Holo) | Antwerp 2022</t>
   </si>
   <si>
-    <t>MP7 | Fade (Field-Tested)</t>
-  </si>
-  <si>
-    <t>Sticker | Great Wave (Holo)</t>
-  </si>
-  <si>
     <t>Sticker | Copenhagen Flames (Holo) | Stockholm 2021</t>
   </si>
   <si>
@@ -265,24 +325,27 @@
     <t>Sticker | Liquid Fire</t>
   </si>
   <si>
+    <t>High Grade</t>
+  </si>
+  <si>
+    <t>AK-47 | Crossfade (Factory New)</t>
+  </si>
+  <si>
     <t>AK-47 | Slate (Minimal Wear)</t>
   </si>
   <si>
-    <t>AK-47 | Crossfade (Factory New)</t>
-  </si>
-  <si>
     <t>Sticker | Team Spirit (Holo) | Stockholm 2021</t>
   </si>
   <si>
     <t>Tec-9 | Brass (Field-Tested)</t>
   </si>
   <si>
+    <t>Dragomir | Sabre</t>
+  </si>
+  <si>
     <t>Maximus | Sabre</t>
   </si>
   <si>
-    <t>Dragomir | Sabre</t>
-  </si>
-  <si>
     <t>XM1014 | Black Tie (Factory New)</t>
   </si>
   <si>
@@ -328,12 +391,18 @@
     <t>MAC-10 | Strats (Factory New)</t>
   </si>
   <si>
+    <t>Consumer Grade</t>
+  </si>
+  <si>
     <t>AWP | Black Nile (Minimal Wear)</t>
   </si>
   <si>
     <t>Sticker | Team Spirit (Holo) | Antwerp 2022</t>
   </si>
   <si>
+    <t>Sticker | Gold Web (Foil)</t>
+  </si>
+  <si>
     <t>Sticker | Imperial Esports (Holo) | Antwerp 2022</t>
   </si>
   <si>
@@ -346,9 +415,6 @@
     <t>P250 | Epicenter (Field-Tested)</t>
   </si>
   <si>
-    <t>Sticker | Gold Web (Foil)</t>
-  </si>
-  <si>
     <t>Sticker | Astralis (Holo) | Stockholm 2021</t>
   </si>
   <si>
@@ -421,10 +487,10 @@
     <t>Sticker | BIG (Holo) | Antwerp 2022</t>
   </si>
   <si>
+    <t>SSG 08 | Ghost Crusader (Minimal Wear)</t>
+  </si>
+  <si>
     <t>Sticker | Broken Fang (Holo)</t>
-  </si>
-  <si>
-    <t>SSG 08 | Ghost Crusader (Minimal Wear)</t>
   </si>
   <si>
     <t>Sticker | forZe eSports (Holo) | Antwerp 2022</t>
@@ -842,11 +908,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="10" width="14" customWidth="1"/>
+    <col min="2" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -876,7 +942,7 @@
         <v>11.534</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -907,10 +973,16 @@
       <c r="J5" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>49</v>
@@ -939,16 +1011,22 @@
       <c r="J6" s="2">
         <f>IF(D6=0,"",(H6-D6)/D6)</f>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B7">
         <v>66</v>
       </c>
       <c r="C7">
-        <v>135.25</v>
+        <v>135.3</v>
       </c>
       <c r="D7">
         <f>C7*$B$3</f>
@@ -971,13 +1049,19 @@
       <c r="J7" s="2">
         <f>IF(D7=0,"",(H7-D7)/D7)</f>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
+        <v>18</v>
+      </c>
+      <c r="L7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B8">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C8">
         <v>119.34</v>
@@ -992,7 +1076,7 @@
         <v>8875.41</v>
       </c>
       <c r="G8">
-        <v>8718.55</v>
+        <v>8737.01</v>
       </c>
       <c r="H8">
         <f>MIN(E8:G8)</f>
@@ -1003,13 +1087,19 @@
       <c r="J8" s="2">
         <f>IF(D8=0,"",(H8-D8)/D8)</f>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" t="s">
+        <v>23</v>
+      </c>
+      <c r="L8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B9">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C9">
         <v>97.13</v>
@@ -1024,7 +1114,7 @@
         <v>7484.18</v>
       </c>
       <c r="G9">
-        <v>7497.1</v>
+        <v>7554.65</v>
       </c>
       <c r="H9">
         <f>MIN(E9:G9)</f>
@@ -1035,16 +1125,22 @@
       <c r="J9" s="2">
         <f>IF(D9=0,"",(H9-D9)/D9)</f>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B10">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C10">
-        <v>88.48</v>
+        <v>88.5</v>
       </c>
       <c r="D10">
         <f>C10*$B$3</f>
@@ -1067,10 +1163,16 @@
       <c r="J10" s="2">
         <f>IF(D10=0,"",(H10-D10)/D10)</f>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B11">
         <v>58</v>
@@ -1099,16 +1201,22 @@
       <c r="J11" s="2">
         <f>IF(D11=0,"",(H11-D11)/D11)</f>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B12">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="C12">
-        <v>80.84</v>
+        <v>81.14</v>
       </c>
       <c r="D12">
         <f>C12*$B$3</f>
@@ -1131,10 +1239,16 @@
       <c r="J12" s="2">
         <f>IF(D12=0,"",(H12-D12)/D12)</f>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B13">
         <v>35</v>
@@ -1163,16 +1277,22 @@
       <c r="J13" s="2">
         <f>IF(D13=0,"",(H13-D13)/D13)</f>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" t="s">
+        <v>18</v>
+      </c>
+      <c r="L13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B14">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C14">
-        <v>59.68</v>
+        <v>59.89</v>
       </c>
       <c r="D14">
         <f>C14*$B$3</f>
@@ -1195,10 +1315,16 @@
       <c r="J14" s="2">
         <f>IF(D14=0,"",(H14-D14)/D14)</f>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="B15">
         <v>299</v>
@@ -1227,10 +1353,16 @@
       <c r="J15" s="2">
         <f>IF(D15=0,"",(H15-D15)/D15)</f>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B16">
         <v>262</v>
@@ -1259,13 +1391,19 @@
       <c r="J16" s="2">
         <f>IF(D16=0,"",(H16-D16)/D16)</f>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>23</v>
+      </c>
+      <c r="L16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B17">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C17">
         <v>57.32</v>
@@ -1280,7 +1418,7 @@
         <v>4394.45</v>
       </c>
       <c r="G17">
-        <v>4354.09</v>
+        <v>4348.32</v>
       </c>
       <c r="H17">
         <f>MIN(E17:G17)</f>
@@ -1291,13 +1429,19 @@
       <c r="J17" s="2">
         <f>IF(D17=0,"",(H17-D17)/D17)</f>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K17" t="s">
+        <v>23</v>
+      </c>
+      <c r="L17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B18">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="C18">
         <v>56.3</v>
@@ -1309,10 +1453,10 @@
         <v>6620.98</v>
       </c>
       <c r="F18">
+        <v>4244.51</v>
+      </c>
+      <c r="G18">
         <v>4152.24</v>
-      </c>
-      <c r="G18">
-        <v>4167</v>
       </c>
       <c r="H18">
         <f>MIN(E18:G18)</f>
@@ -1323,10 +1467,16 @@
       <c r="J18" s="2">
         <f>IF(D18=0,"",(H18-D18)/D18)</f>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K18" t="s">
+        <v>30</v>
+      </c>
+      <c r="L18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B19">
         <v>274</v>
@@ -1355,10 +1505,16 @@
       <c r="J19" s="2">
         <f>IF(D19=0,"",(H19-D19)/D19)</f>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K19" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B20">
         <v>75</v>
@@ -1387,10 +1543,16 @@
       <c r="J20" s="2">
         <f>IF(D20=0,"",(H20-D20)/D20)</f>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K20" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="B21">
         <v>72</v>
@@ -1419,13 +1581,19 @@
       <c r="J21" s="2">
         <f>IF(D21=0,"",(H21-D21)/D21)</f>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B22">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C22">
         <v>48.6</v>
@@ -1451,10 +1619,16 @@
       <c r="J22" s="2">
         <f>IF(D22=0,"",(H22-D22)/D22)</f>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" t="s">
+        <v>26</v>
+      </c>
+      <c r="L22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B23">
         <v>60</v>
@@ -1483,13 +1657,19 @@
       <c r="J23" s="2">
         <f>IF(D23=0,"",(H23-D23)/D23)</f>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" t="s">
+        <v>23</v>
+      </c>
+      <c r="L23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B24">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C24">
         <v>48.45</v>
@@ -1515,10 +1695,16 @@
       <c r="J24" s="2">
         <f>IF(D24=0,"",(H24-D24)/D24)</f>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K24" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B25">
         <v>110</v>
@@ -1547,10 +1733,16 @@
       <c r="J25" s="2">
         <f>IF(D25=0,"",(H25-D25)/D25)</f>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K25" t="s">
+        <v>23</v>
+      </c>
+      <c r="L25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B26">
         <v>66</v>
@@ -1579,10 +1771,16 @@
       <c r="J26" s="2">
         <f>IF(D26=0,"",(H26-D26)/D26)</f>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K26" t="s">
+        <v>23</v>
+      </c>
+      <c r="L26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B27">
         <v>94</v>
@@ -1611,16 +1809,22 @@
       <c r="J27" s="2">
         <f>IF(D27=0,"",(H27-D27)/D27)</f>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K27" t="s">
+        <v>30</v>
+      </c>
+      <c r="L27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B28">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C28">
-        <v>32.57</v>
+        <v>32.66</v>
       </c>
       <c r="D28">
         <f>C28*$B$3</f>
@@ -1643,16 +1847,22 @@
       <c r="J28" s="2">
         <f>IF(D28=0,"",(H28-D28)/D28)</f>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K28" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B29">
         <v>137</v>
       </c>
       <c r="C29">
-        <v>32.05</v>
+        <v>31.67</v>
       </c>
       <c r="D29">
         <f>C29*$B$3</f>
@@ -1675,16 +1885,22 @@
       <c r="J29" s="2">
         <f>IF(D29=0,"",(H29-D29)/D29)</f>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K29" t="s">
+        <v>26</v>
+      </c>
+      <c r="L29" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B30">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C30">
-        <v>29.46</v>
+        <v>29.48</v>
       </c>
       <c r="D30">
         <f>C30*$B$3</f>
@@ -1707,10 +1923,16 @@
       <c r="J30" s="2">
         <f>IF(D30=0,"",(H30-D30)/D30)</f>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K30" t="s">
+        <v>30</v>
+      </c>
+      <c r="L30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B31">
         <v>229</v>
@@ -1739,16 +1961,22 @@
       <c r="J31" s="2">
         <f>IF(D31=0,"",(H31-D31)/D31)</f>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K31" t="s">
+        <v>18</v>
+      </c>
+      <c r="L31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="B32">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C32">
-        <v>23.23</v>
+        <v>23.24</v>
       </c>
       <c r="D32">
         <f>C32*$B$3</f>
@@ -1771,10 +1999,16 @@
       <c r="J32" s="2">
         <f>IF(D32=0,"",(H32-D32)/D32)</f>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K32" t="s">
+        <v>52</v>
+      </c>
+      <c r="L32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="B33">
         <v>149</v>
@@ -1803,16 +2037,22 @@
       <c r="J33" s="2">
         <f>IF(D33=0,"",(H33-D33)/D33)</f>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K33" t="s">
+        <v>26</v>
+      </c>
+      <c r="L33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B34">
         <v>80</v>
       </c>
       <c r="C34">
-        <v>19.8</v>
+        <v>19.79</v>
       </c>
       <c r="D34">
         <f>C34*$B$3</f>
@@ -1835,13 +2075,19 @@
       <c r="J34" s="2">
         <f>IF(D34=0,"",(H34-D34)/D34)</f>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K34" t="s">
+        <v>26</v>
+      </c>
+      <c r="L34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="B35">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C35">
         <v>19.51</v>
@@ -1867,13 +2113,19 @@
       <c r="J35" s="2">
         <f>IF(D35=0,"",(H35-D35)/D35)</f>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K35" t="s">
+        <v>23</v>
+      </c>
+      <c r="L35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B36">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C36">
         <v>18.95</v>
@@ -1899,13 +2151,19 @@
       <c r="J36" s="2">
         <f>IF(D36=0,"",(H36-D36)/D36)</f>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K36" t="s">
+        <v>58</v>
+      </c>
+      <c r="L36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B37">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C37">
         <v>18.84</v>
@@ -1931,16 +2189,22 @@
       <c r="J37" s="2">
         <f>IF(D37=0,"",(H37-D37)/D37)</f>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K37" t="s">
+        <v>26</v>
+      </c>
+      <c r="L37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B38">
         <v>79</v>
       </c>
       <c r="C38">
-        <v>15.43</v>
+        <v>15.41</v>
       </c>
       <c r="D38">
         <f>C38*$B$3</f>
@@ -1963,10 +2227,16 @@
       <c r="J38" s="2">
         <f>IF(D38=0,"",(H38-D38)/D38)</f>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K38" t="s">
+        <v>23</v>
+      </c>
+      <c r="L38" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B39">
         <v>47</v>
@@ -1995,10 +2265,16 @@
       <c r="J39" s="2">
         <f>IF(D39=0,"",(H39-D39)/D39)</f>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K39" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="B40">
         <v>26</v>
@@ -2027,10 +2303,16 @@
       <c r="J40" s="2">
         <f>IF(D40=0,"",(H40-D40)/D40)</f>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K40" t="s">
+        <v>58</v>
+      </c>
+      <c r="L40" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="B41">
         <v>67</v>
@@ -2059,13 +2341,19 @@
       <c r="J41" s="2">
         <f>IF(D41=0,"",(H41-D41)/D41)</f>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K41" t="s">
+        <v>64</v>
+      </c>
+      <c r="L41" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="B42">
-        <v>1738</v>
+        <v>1735</v>
       </c>
       <c r="C42">
         <v>13.49</v>
@@ -2091,10 +2379,16 @@
       <c r="J42" s="2">
         <f>IF(D42=0,"",(H42-D42)/D42)</f>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K42" t="s">
+        <v>52</v>
+      </c>
+      <c r="L42" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="B43">
         <v>60</v>
@@ -2123,13 +2417,19 @@
       <c r="J43" s="2">
         <f>IF(D43=0,"",(H43-D43)/D43)</f>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K43" t="s">
+        <v>23</v>
+      </c>
+      <c r="L43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B44">
-        <v>1424</v>
+        <v>1420</v>
       </c>
       <c r="C44">
         <v>13.01</v>
@@ -2155,10 +2455,16 @@
       <c r="J44" s="2">
         <f>IF(D44=0,"",(H44-D44)/D44)</f>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K44" t="s">
+        <v>52</v>
+      </c>
+      <c r="L44" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="B45">
         <v>3</v>
@@ -2187,10 +2493,16 @@
       <c r="J45" s="2">
         <f>IF(D45=0,"",(H45-D45)/D45)</f>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K45" t="s">
+        <v>64</v>
+      </c>
+      <c r="L45" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="B46">
         <v>371</v>
@@ -2219,10 +2531,16 @@
       <c r="J46" s="2">
         <f>IF(D46=0,"",(H46-D46)/D46)</f>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K46" t="s">
+        <v>26</v>
+      </c>
+      <c r="L46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="B47">
         <v>95</v>
@@ -2251,10 +2569,16 @@
       <c r="J47" s="2">
         <f>IF(D47=0,"",(H47-D47)/D47)</f>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K47" t="s">
+        <v>26</v>
+      </c>
+      <c r="L47" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="B48">
         <v>176</v>
@@ -2283,10 +2607,16 @@
       <c r="J48" s="2">
         <f>IF(D48=0,"",(H48-D48)/D48)</f>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K48" t="s">
+        <v>30</v>
+      </c>
+      <c r="L48" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="B49">
         <v>1768</v>
@@ -2315,13 +2645,19 @@
       <c r="J49" s="2">
         <f>IF(D49=0,"",(H49-D49)/D49)</f>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K49" t="s">
+        <v>52</v>
+      </c>
+      <c r="L49" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="B50">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C50">
         <v>10.58</v>
@@ -2347,10 +2683,16 @@
       <c r="J50" s="2">
         <f>IF(D50=0,"",(H50-D50)/D50)</f>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K50" t="s">
+        <v>23</v>
+      </c>
+      <c r="L50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B51">
         <v>202</v>
@@ -2379,10 +2721,16 @@
       <c r="J51" s="2">
         <f>IF(D51=0,"",(H51-D51)/D51)</f>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K51" t="s">
+        <v>64</v>
+      </c>
+      <c r="L51" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B52">
         <v>84</v>
@@ -2411,13 +2759,19 @@
       <c r="J52" s="2">
         <f>IF(D52=0,"",(H52-D52)/D52)</f>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K52" t="s">
+        <v>23</v>
+      </c>
+      <c r="L52" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="B53">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C53">
         <v>10.19</v>
@@ -2443,10 +2797,16 @@
       <c r="J53" s="2">
         <f>IF(D53=0,"",(H53-D53)/D53)</f>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K53" t="s">
+        <v>26</v>
+      </c>
+      <c r="L53" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="B54">
         <v>100</v>
@@ -2475,10 +2835,16 @@
       <c r="J54" s="2">
         <f>IF(D54=0,"",(H54-D54)/D54)</f>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K54" t="s">
+        <v>23</v>
+      </c>
+      <c r="L54" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="B55">
         <v>493</v>
@@ -2507,10 +2873,16 @@
       <c r="J55" s="2">
         <f>IF(D55=0,"",(H55-D55)/D55)</f>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K55" t="s">
+        <v>23</v>
+      </c>
+      <c r="L55" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="B56">
         <v>1313</v>
@@ -2539,13 +2911,19 @@
       <c r="J56" s="2">
         <f>IF(D56=0,"",(H56-D56)/D56)</f>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K56" t="s">
+        <v>52</v>
+      </c>
+      <c r="L56" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="B57">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="C57">
         <v>9.7</v>
@@ -2571,10 +2949,16 @@
       <c r="J57" s="2">
         <f>IF(D57=0,"",(H57-D57)/D57)</f>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K57" t="s">
+        <v>52</v>
+      </c>
+      <c r="L57" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="B58">
         <v>95</v>
@@ -2603,13 +2987,19 @@
       <c r="J58" s="2">
         <f>IF(D58=0,"",(H58-D58)/D58)</f>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K58" t="s">
+        <v>26</v>
+      </c>
+      <c r="L58" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="B59">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C59">
         <v>8.92</v>
@@ -2635,10 +3025,16 @@
       <c r="J59" s="2">
         <f>IF(D59=0,"",(H59-D59)/D59)</f>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K59" t="s">
+        <v>30</v>
+      </c>
+      <c r="L59" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="B60">
         <v>688</v>
@@ -2667,10 +3063,16 @@
       <c r="J60" s="2">
         <f>IF(D60=0,"",(H60-D60)/D60)</f>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K60" t="s">
+        <v>52</v>
+      </c>
+      <c r="L60" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="B61">
         <v>561</v>
@@ -2699,28 +3101,34 @@
       <c r="J61" s="2">
         <f>IF(D61=0,"",(H61-D61)/D61)</f>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K61" t="s">
+        <v>18</v>
+      </c>
+      <c r="L61" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="B62">
-        <v>100</v>
+        <v>189</v>
       </c>
       <c r="C62">
-        <v>8.28</v>
+        <v>8.29</v>
       </c>
       <c r="D62">
         <f>C62*$B$3</f>
       </c>
       <c r="E62">
-        <v>934.83</v>
+        <v>910.49</v>
       </c>
       <c r="F62">
-        <v>678.2</v>
+        <v>631.26</v>
       </c>
       <c r="G62">
-        <v>632.06</v>
+        <v>611.3</v>
       </c>
       <c r="H62">
         <f>MIN(E62:G62)</f>
@@ -2731,28 +3139,34 @@
       <c r="J62" s="2">
         <f>IF(D62=0,"",(H62-D62)/D62)</f>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K62" t="s">
+        <v>18</v>
+      </c>
+      <c r="L62" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="B63">
-        <v>190</v>
+        <v>25</v>
       </c>
       <c r="C63">
-        <v>8.27</v>
+        <v>8.25</v>
       </c>
       <c r="D63">
         <f>C63*$B$3</f>
       </c>
       <c r="E63">
-        <v>910.49</v>
+        <v>938.87</v>
       </c>
       <c r="F63">
-        <v>631.26</v>
+        <v>609</v>
       </c>
       <c r="G63">
-        <v>611.3</v>
+        <v>629.3</v>
       </c>
       <c r="H63">
         <f>MIN(E63:G63)</f>
@@ -2763,13 +3177,19 @@
       <c r="J63" s="2">
         <f>IF(D63=0,"",(H63-D63)/D63)</f>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K63" t="s">
+        <v>64</v>
+      </c>
+      <c r="L63" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B64">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C64">
         <v>8.25</v>
@@ -2778,13 +3198,13 @@
         <f>C64*$B$3</f>
       </c>
       <c r="E64">
-        <v>938.87</v>
+        <v>934.83</v>
       </c>
       <c r="F64">
-        <v>609</v>
+        <v>678.2</v>
       </c>
       <c r="G64">
-        <v>629.3</v>
+        <v>632.06</v>
       </c>
       <c r="H64">
         <f>MIN(E64:G64)</f>
@@ -2795,10 +3215,16 @@
       <c r="J64" s="2">
         <f>IF(D64=0,"",(H64-D64)/D64)</f>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K64" t="s">
+        <v>64</v>
+      </c>
+      <c r="L64" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="B65">
         <v>268</v>
@@ -2827,10 +3253,16 @@
       <c r="J65" s="2">
         <f>IF(D65=0,"",(H65-D65)/D65)</f>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K65" t="s">
+        <v>64</v>
+      </c>
+      <c r="L65" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="B66">
         <v>131</v>
@@ -2859,16 +3291,22 @@
       <c r="J66" s="2">
         <f>IF(D66=0,"",(H66-D66)/D66)</f>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K66" t="s">
+        <v>26</v>
+      </c>
+      <c r="L66" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B67">
-        <v>846</v>
+        <v>842</v>
       </c>
       <c r="C67">
-        <v>7.98</v>
+        <v>7.99</v>
       </c>
       <c r="D67">
         <f>C67*$B$3</f>
@@ -2891,13 +3329,19 @@
       <c r="J67" s="2">
         <f>IF(D67=0,"",(H67-D67)/D67)</f>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K67" t="s">
+        <v>52</v>
+      </c>
+      <c r="L67" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="B68">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="C68">
         <v>7.88</v>
@@ -2923,13 +3367,19 @@
       <c r="J68" s="2">
         <f>IF(D68=0,"",(H68-D68)/D68)</f>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K68" t="s">
+        <v>52</v>
+      </c>
+      <c r="L68" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="B69">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="C69">
         <v>7.83</v>
@@ -2955,13 +3405,19 @@
       <c r="J69" s="2">
         <f>IF(D69=0,"",(H69-D69)/D69)</f>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K69" t="s">
+        <v>52</v>
+      </c>
+      <c r="L69" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B70">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="C70">
         <v>7.82</v>
@@ -2987,10 +3443,16 @@
       <c r="J70" s="2">
         <f>IF(D70=0,"",(H70-D70)/D70)</f>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K70" t="s">
+        <v>52</v>
+      </c>
+      <c r="L70" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B71">
         <v>143</v>
@@ -3019,13 +3481,19 @@
       <c r="J71" s="2">
         <f>IF(D71=0,"",(H71-D71)/D71)</f>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K71" t="s">
+        <v>64</v>
+      </c>
+      <c r="L71" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B72">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="C72">
         <v>7.39</v>
@@ -3051,10 +3519,16 @@
       <c r="J72" s="2">
         <f>IF(D72=0,"",(H72-D72)/D72)</f>
       </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K72" t="s">
+        <v>52</v>
+      </c>
+      <c r="L72" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B73">
         <v>207</v>
@@ -3083,10 +3557,16 @@
       <c r="J73" s="2">
         <f>IF(D73=0,"",(H73-D73)/D73)</f>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K73" t="s">
+        <v>64</v>
+      </c>
+      <c r="L73" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B74">
         <v>8</v>
@@ -3115,28 +3595,34 @@
       <c r="J74" s="2">
         <f>IF(D74=0,"",(H74-D74)/D74)</f>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K74" t="s">
+        <v>64</v>
+      </c>
+      <c r="L74" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="B75">
-        <v>1326</v>
+        <v>394</v>
       </c>
       <c r="C75">
-        <v>6.84</v>
+        <v>6.82</v>
       </c>
       <c r="D75">
         <f>C75*$B$3</f>
       </c>
       <c r="E75">
-        <v>809.57</v>
+        <v>765.4</v>
       </c>
       <c r="F75">
-        <v>513.26</v>
+        <v>484.43</v>
       </c>
       <c r="G75">
-        <v>514.42</v>
+        <v>480.97</v>
       </c>
       <c r="H75">
         <f>MIN(E75:G75)</f>
@@ -3147,28 +3633,34 @@
       <c r="J75" s="2">
         <f>IF(D75=0,"",(H75-D75)/D75)</f>
       </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K75" t="s">
+        <v>26</v>
+      </c>
+      <c r="L75" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="B76">
-        <v>389</v>
+        <v>1326</v>
       </c>
       <c r="C76">
-        <v>6.82</v>
+        <v>6.78</v>
       </c>
       <c r="D76">
         <f>C76*$B$3</f>
       </c>
       <c r="E76">
-        <v>765.4</v>
+        <v>809.57</v>
       </c>
       <c r="F76">
-        <v>484.43</v>
+        <v>513.26</v>
       </c>
       <c r="G76">
-        <v>480.97</v>
+        <v>514.42</v>
       </c>
       <c r="H76">
         <f>MIN(E76:G76)</f>
@@ -3179,10 +3671,16 @@
       <c r="J76" s="2">
         <f>IF(D76=0,"",(H76-D76)/D76)</f>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K76" t="s">
+        <v>26</v>
+      </c>
+      <c r="L76" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="B77">
         <v>59</v>
@@ -3211,10 +3709,16 @@
       <c r="J77" s="2">
         <f>IF(D77=0,"",(H77-D77)/D77)</f>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K77" t="s">
+        <v>64</v>
+      </c>
+      <c r="L77" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="B78">
         <v>77</v>
@@ -3243,28 +3747,34 @@
       <c r="J78" s="2">
         <f>IF(D78=0,"",(H78-D78)/D78)</f>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K78" t="s">
+        <v>23</v>
+      </c>
+      <c r="L78" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="B79">
-        <v>1194</v>
+        <v>940</v>
       </c>
       <c r="C79">
-        <v>6.44</v>
+        <v>6.45</v>
       </c>
       <c r="D79">
         <f>C79*$B$3</f>
       </c>
       <c r="E79">
-        <v>768.51</v>
+        <v>784.31</v>
       </c>
       <c r="F79">
-        <v>475.32</v>
+        <v>479.81</v>
       </c>
       <c r="G79">
-        <v>480.74</v>
+        <v>473.93</v>
       </c>
       <c r="H79">
         <f>MIN(E79:G79)</f>
@@ -3275,13 +3785,19 @@
       <c r="J79" s="2">
         <f>IF(D79=0,"",(H79-D79)/D79)</f>
       </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K79" t="s">
+        <v>52</v>
+      </c>
+      <c r="L79" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="B80">
-        <v>940</v>
+        <v>1193</v>
       </c>
       <c r="C80">
         <v>6.44</v>
@@ -3290,13 +3806,13 @@
         <f>C80*$B$3</f>
       </c>
       <c r="E80">
-        <v>784.31</v>
+        <v>768.51</v>
       </c>
       <c r="F80">
-        <v>479.81</v>
+        <v>475.32</v>
       </c>
       <c r="G80">
-        <v>473.93</v>
+        <v>480.74</v>
       </c>
       <c r="H80">
         <f>MIN(E80:G80)</f>
@@ -3307,10 +3823,16 @@
       <c r="J80" s="2">
         <f>IF(D80=0,"",(H80-D80)/D80)</f>
       </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K80" t="s">
+        <v>52</v>
+      </c>
+      <c r="L80" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B81">
         <v>72</v>
@@ -3339,10 +3861,16 @@
       <c r="J81" s="2">
         <f>IF(D81=0,"",(H81-D81)/D81)</f>
       </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K81" t="s">
+        <v>58</v>
+      </c>
+      <c r="L81" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="B82">
         <v>104</v>
@@ -3371,10 +3899,16 @@
       <c r="J82" s="2">
         <f>IF(D82=0,"",(H82-D82)/D82)</f>
       </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K82" t="s">
+        <v>64</v>
+      </c>
+      <c r="L82" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="B83">
         <v>227</v>
@@ -3403,10 +3937,16 @@
       <c r="J83" s="2">
         <f>IF(D83=0,"",(H83-D83)/D83)</f>
       </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K83" t="s">
+        <v>64</v>
+      </c>
+      <c r="L83" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="B84">
         <v>72</v>
@@ -3435,10 +3975,16 @@
       <c r="J84" s="2">
         <f>IF(D84=0,"",(H84-D84)/D84)</f>
       </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K84" t="s">
+        <v>64</v>
+      </c>
+      <c r="L84" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="B85">
         <v>123</v>
@@ -3467,10 +4013,16 @@
       <c r="J85" s="2">
         <f>IF(D85=0,"",(H85-D85)/D85)</f>
       </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K85" t="s">
+        <v>64</v>
+      </c>
+      <c r="L85" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="B86">
         <v>112</v>
@@ -3499,10 +4051,16 @@
       <c r="J86" s="2">
         <f>IF(D86=0,"",(H86-D86)/D86)</f>
       </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K86" t="s">
+        <v>64</v>
+      </c>
+      <c r="L86" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="B87">
         <v>97</v>
@@ -3531,10 +4089,16 @@
       <c r="J87" s="2">
         <f>IF(D87=0,"",(H87-D87)/D87)</f>
       </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K87" t="s">
+        <v>64</v>
+      </c>
+      <c r="L87" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="B88">
         <v>136</v>
@@ -3563,10 +4127,16 @@
       <c r="J88" s="2">
         <f>IF(D88=0,"",(H88-D88)/D88)</f>
       </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K88" t="s">
+        <v>64</v>
+      </c>
+      <c r="L88" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="B89">
         <v>155</v>
@@ -3595,10 +4165,16 @@
       <c r="J89" s="2">
         <f>IF(D89=0,"",(H89-D89)/D89)</f>
       </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K89" t="s">
+        <v>23</v>
+      </c>
+      <c r="L89" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="B90">
         <v>511</v>
@@ -3627,10 +4203,16 @@
       <c r="J90" s="2">
         <f>IF(D90=0,"",(H90-D90)/D90)</f>
       </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K90" t="s">
+        <v>64</v>
+      </c>
+      <c r="L90" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="B91">
         <v>122</v>
@@ -3659,10 +4241,16 @@
       <c r="J91" s="2">
         <f>IF(D91=0,"",(H91-D91)/D91)</f>
       </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K91" t="s">
+        <v>64</v>
+      </c>
+      <c r="L91" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="B92">
         <v>175</v>
@@ -3691,13 +4279,19 @@
       <c r="J92" s="2">
         <f>IF(D92=0,"",(H92-D92)/D92)</f>
       </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K92" t="s">
+        <v>64</v>
+      </c>
+      <c r="L92" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="B93">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C93">
         <v>5.31</v>
@@ -3723,10 +4317,16 @@
       <c r="J93" s="2">
         <f>IF(D93=0,"",(H93-D93)/D93)</f>
       </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L93" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="B94">
         <v>29</v>
@@ -3755,10 +4355,16 @@
       <c r="J94" s="2">
         <f>IF(D94=0,"",(H94-D94)/D94)</f>
       </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K94" t="s">
+        <v>23</v>
+      </c>
+      <c r="L94" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="B95">
         <v>62</v>
@@ -3787,13 +4393,19 @@
       <c r="J95" s="2">
         <f>IF(D95=0,"",(H95-D95)/D95)</f>
       </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K95" t="s">
+        <v>18</v>
+      </c>
+      <c r="L95" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="B96">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C96">
         <v>4.96</v>
@@ -3819,10 +4431,16 @@
       <c r="J96" s="2">
         <f>IF(D96=0,"",(H96-D96)/D96)</f>
       </c>
-    </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K96" t="s">
+        <v>30</v>
+      </c>
+      <c r="L96" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="B97">
         <v>73</v>
@@ -3851,28 +4469,34 @@
       <c r="J97" s="2">
         <f>IF(D97=0,"",(H97-D97)/D97)</f>
       </c>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K97" t="s">
+        <v>64</v>
+      </c>
+      <c r="L97" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="B98">
-        <v>120</v>
+        <v>159</v>
       </c>
       <c r="C98">
-        <v>4.81</v>
+        <v>4.86</v>
       </c>
       <c r="D98">
         <f>C98*$B$3</f>
       </c>
       <c r="E98">
-        <v>588.81</v>
+        <v>562.74</v>
       </c>
       <c r="F98">
-        <v>411.07</v>
+        <v>344.75</v>
       </c>
       <c r="G98">
-        <v>379.47</v>
+        <v>322.95</v>
       </c>
       <c r="H98">
         <f>MIN(E98:G98)</f>
@@ -3883,28 +4507,34 @@
       <c r="J98" s="2">
         <f>IF(D98=0,"",(H98-D98)/D98)</f>
       </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K98" t="s">
+        <v>64</v>
+      </c>
+      <c r="L98" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="B99">
-        <v>618</v>
+        <v>121</v>
       </c>
       <c r="C99">
-        <v>4.77</v>
+        <v>4.81</v>
       </c>
       <c r="D99">
         <f>C99*$B$3</f>
       </c>
       <c r="E99">
-        <v>507.61</v>
+        <v>588.81</v>
       </c>
       <c r="F99">
-        <v>356.75</v>
+        <v>411.07</v>
       </c>
       <c r="G99">
-        <v>364.24</v>
+        <v>379.47</v>
       </c>
       <c r="H99">
         <f>MIN(E99:G99)</f>
@@ -3915,28 +4545,34 @@
       <c r="J99" s="2">
         <f>IF(D99=0,"",(H99-D99)/D99)</f>
       </c>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K99" t="s">
+        <v>64</v>
+      </c>
+      <c r="L99" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="B100">
-        <v>78</v>
+        <v>619</v>
       </c>
       <c r="C100">
-        <v>4.71</v>
+        <v>4.77</v>
       </c>
       <c r="D100">
         <f>C100*$B$3</f>
       </c>
       <c r="E100">
-        <v>599.88</v>
+        <v>507.61</v>
       </c>
       <c r="F100">
-        <v>373.59</v>
+        <v>356.75</v>
       </c>
       <c r="G100">
-        <v>380.62</v>
+        <v>364.24</v>
       </c>
       <c r="H100">
         <f>MIN(E100:G100)</f>
@@ -3947,28 +4583,34 @@
       <c r="J100" s="2">
         <f>IF(D100=0,"",(H100-D100)/D100)</f>
       </c>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K100" t="s">
+        <v>23</v>
+      </c>
+      <c r="L100" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="B101">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C101">
-        <v>4.69</v>
+        <v>4.71</v>
       </c>
       <c r="D101">
         <f>C101*$B$3</f>
       </c>
       <c r="E101">
-        <v>535.18</v>
+        <v>599.88</v>
       </c>
       <c r="F101">
-        <v>334.49</v>
+        <v>373.59</v>
       </c>
       <c r="G101">
-        <v>373.59</v>
+        <v>380.62</v>
       </c>
       <c r="H101">
         <f>MIN(E101:G101)</f>
@@ -3979,28 +4621,34 @@
       <c r="J101" s="2">
         <f>IF(D101=0,"",(H101-D101)/D101)</f>
       </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K101" t="s">
+        <v>64</v>
+      </c>
+      <c r="L101" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="B102">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="C102">
-        <v>4.66</v>
+        <v>4.69</v>
       </c>
       <c r="D102">
         <f>C102*$B$3</f>
       </c>
       <c r="E102">
-        <v>562.74</v>
+        <v>535.18</v>
       </c>
       <c r="F102">
-        <v>344.75</v>
+        <v>334.49</v>
       </c>
       <c r="G102">
-        <v>322.95</v>
+        <v>373.59</v>
       </c>
       <c r="H102">
         <f>MIN(E102:G102)</f>
@@ -4011,10 +4659,16 @@
       <c r="J102" s="2">
         <f>IF(D102=0,"",(H102-D102)/D102)</f>
       </c>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K102" t="s">
+        <v>23</v>
+      </c>
+      <c r="L102" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="B103">
         <v>55</v>
@@ -4043,10 +4697,16 @@
       <c r="J103" s="2">
         <f>IF(D103=0,"",(H103-D103)/D103)</f>
       </c>
-    </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K103" t="s">
+        <v>64</v>
+      </c>
+      <c r="L103" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="B104">
         <v>25</v>
@@ -4075,10 +4735,16 @@
       <c r="J104" s="2">
         <f>IF(D104=0,"",(H104-D104)/D104)</f>
       </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K104" t="s">
+        <v>64</v>
+      </c>
+      <c r="L104" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="B105">
         <v>110</v>
@@ -4107,10 +4773,16 @@
       <c r="J105" s="2">
         <f>IF(D105=0,"",(H105-D105)/D105)</f>
       </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K105" t="s">
+        <v>64</v>
+      </c>
+      <c r="L105" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="B106">
         <v>42</v>
@@ -4139,10 +4811,16 @@
       <c r="J106" s="2">
         <f>IF(D106=0,"",(H106-D106)/D106)</f>
       </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K106" t="s">
+        <v>64</v>
+      </c>
+      <c r="L106" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="B107">
         <v>101</v>
@@ -4171,16 +4849,22 @@
       <c r="J107" s="2">
         <f>IF(D107=0,"",(H107-D107)/D107)</f>
       </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K107" t="s">
+        <v>64</v>
+      </c>
+      <c r="L107" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="B108">
-        <v>2417</v>
+        <v>2419</v>
       </c>
       <c r="C108">
-        <v>4.35</v>
+        <v>4.31</v>
       </c>
       <c r="D108">
         <f>C108*$B$3</f>
@@ -4203,10 +4887,16 @@
       <c r="J108" s="2">
         <f>IF(D108=0,"",(H108-D108)/D108)</f>
       </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K108" t="s">
+        <v>26</v>
+      </c>
+      <c r="L108" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="B109">
         <v>54</v>
@@ -4235,10 +4925,16 @@
       <c r="J109" s="2">
         <f>IF(D109=0,"",(H109-D109)/D109)</f>
       </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K109" t="s">
+        <v>64</v>
+      </c>
+      <c r="L109" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="B110">
         <v>123</v>
@@ -4267,13 +4963,19 @@
       <c r="J110" s="2">
         <f>IF(D110=0,"",(H110-D110)/D110)</f>
       </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K110" t="s">
+        <v>64</v>
+      </c>
+      <c r="L110" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="B111">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C111">
         <v>3.86</v>
@@ -4299,10 +5001,16 @@
       <c r="J111" s="2">
         <f>IF(D111=0,"",(H111-D111)/D111)</f>
       </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K111" t="s">
+        <v>26</v>
+      </c>
+      <c r="L111" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="B112">
         <v>360</v>
@@ -4331,10 +5039,16 @@
       <c r="J112" s="2">
         <f>IF(D112=0,"",(H112-D112)/D112)</f>
       </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K112" t="s">
+        <v>64</v>
+      </c>
+      <c r="L112" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="B113">
         <v>365</v>
@@ -4349,7 +5063,7 @@
         <v>405.19</v>
       </c>
       <c r="F113">
-        <v>288.23</v>
+        <v>292.39</v>
       </c>
       <c r="G113">
         <v>276.82</v>
@@ -4363,10 +5077,16 @@
       <c r="J113" s="2">
         <f>IF(D113=0,"",(H113-D113)/D113)</f>
       </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K113" t="s">
+        <v>26</v>
+      </c>
+      <c r="L113" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="B114">
         <v>128</v>
@@ -4395,10 +5115,16 @@
       <c r="J114" s="2">
         <f>IF(D114=0,"",(H114-D114)/D114)</f>
       </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K114" t="s">
+        <v>64</v>
+      </c>
+      <c r="L114" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="B115">
         <v>48</v>
@@ -4427,10 +5153,16 @@
       <c r="J115" s="2">
         <f>IF(D115=0,"",(H115-D115)/D115)</f>
       </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K115" t="s">
+        <v>58</v>
+      </c>
+      <c r="L115" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="B116">
         <v>77</v>
@@ -4459,16 +5191,22 @@
       <c r="J116" s="2">
         <f>IF(D116=0,"",(H116-D116)/D116)</f>
       </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K116" t="s">
+        <v>64</v>
+      </c>
+      <c r="L116" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="B117">
         <v>78</v>
       </c>
       <c r="C117">
-        <v>3.41</v>
+        <v>3.39</v>
       </c>
       <c r="D117">
         <f>C117*$B$3</f>
@@ -4491,13 +5229,19 @@
       <c r="J117" s="2">
         <f>IF(D117=0,"",(H117-D117)/D117)</f>
       </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K117" t="s">
+        <v>23</v>
+      </c>
+      <c r="L117" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="B118">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C118">
         <v>3.35</v>
@@ -4523,10 +5267,16 @@
       <c r="J118" s="2">
         <f>IF(D118=0,"",(H118-D118)/D118)</f>
       </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K118" t="s">
+        <v>23</v>
+      </c>
+      <c r="L118" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="B119">
         <v>247</v>
@@ -4555,13 +5305,19 @@
       <c r="J119" s="2">
         <f>IF(D119=0,"",(H119-D119)/D119)</f>
       </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K119" t="s">
+        <v>64</v>
+      </c>
+      <c r="L119" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="B120">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="C120">
         <v>3.17</v>
@@ -4587,13 +5343,19 @@
       <c r="J120" s="2">
         <f>IF(D120=0,"",(H120-D120)/D120)</f>
       </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K120" t="s">
+        <v>23</v>
+      </c>
+      <c r="L120" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="B121">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C121">
         <v>3.16</v>
@@ -4619,10 +5381,16 @@
       <c r="J121" s="2">
         <f>IF(D121=0,"",(H121-D121)/D121)</f>
       </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K121" t="s">
+        <v>26</v>
+      </c>
+      <c r="L121" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="B122">
         <v>43</v>
@@ -4651,10 +5419,16 @@
       <c r="J122" s="2">
         <f>IF(D122=0,"",(H122-D122)/D122)</f>
       </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K122" t="s">
+        <v>23</v>
+      </c>
+      <c r="L122" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="B123">
         <v>117</v>
@@ -4683,13 +5457,19 @@
       <c r="J123" s="2">
         <f>IF(D123=0,"",(H123-D123)/D123)</f>
       </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K123" t="s">
+        <v>23</v>
+      </c>
+      <c r="L123" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="B124">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C124">
         <v>2.88</v>
@@ -4715,10 +5495,16 @@
       <c r="J124" s="2">
         <f>IF(D124=0,"",(H124-D124)/D124)</f>
       </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K124" t="s">
+        <v>64</v>
+      </c>
+      <c r="L124" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="B125">
         <v>36</v>
@@ -4747,16 +5533,22 @@
       <c r="J125" s="2">
         <f>IF(D125=0,"",(H125-D125)/D125)</f>
       </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K125" t="s">
+        <v>58</v>
+      </c>
+      <c r="L125" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>135</v>
+        <v>157</v>
       </c>
       <c r="B126">
         <v>67</v>
       </c>
       <c r="C126">
-        <v>2.27</v>
+        <v>2.26</v>
       </c>
       <c r="D126">
         <f>C126*$B$3</f>
@@ -4779,13 +5571,19 @@
       <c r="J126" s="2">
         <f>IF(D126=0,"",(H126-D126)/D126)</f>
       </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K126" t="s">
+        <v>64</v>
+      </c>
+      <c r="L126" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
+        <v>158</v>
+      </c>
+      <c r="B127">
         <v>136</v>
-      </c>
-      <c r="B127">
-        <v>106</v>
       </c>
       <c r="C127">
         <v>2.25</v>
@@ -4794,13 +5592,13 @@
         <f>C127*$B$3</f>
       </c>
       <c r="E127">
-        <v>295.62</v>
+        <v>285.35</v>
       </c>
       <c r="F127">
-        <v>174.86</v>
+        <v>177.28</v>
       </c>
       <c r="G127">
-        <v>177.62</v>
+        <v>165.97</v>
       </c>
       <c r="H127">
         <f>MIN(E127:G127)</f>
@@ -4811,13 +5609,19 @@
       <c r="J127" s="2">
         <f>IF(D127=0,"",(H127-D127)/D127)</f>
       </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K127" t="s">
+        <v>30</v>
+      </c>
+      <c r="L127" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="B128">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="C128">
         <v>2.25</v>
@@ -4826,13 +5630,13 @@
         <f>C128*$B$3</f>
       </c>
       <c r="E128">
-        <v>285.35</v>
+        <v>295.62</v>
       </c>
       <c r="F128">
-        <v>177.28</v>
+        <v>174.86</v>
       </c>
       <c r="G128">
-        <v>165.97</v>
+        <v>177.62</v>
       </c>
       <c r="H128">
         <f>MIN(E128:G128)</f>
@@ -4843,10 +5647,16 @@
       <c r="J128" s="2">
         <f>IF(D128=0,"",(H128-D128)/D128)</f>
       </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K128" t="s">
+        <v>64</v>
+      </c>
+      <c r="L128" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="B129">
         <v>20</v>
@@ -4875,10 +5685,16 @@
       <c r="J129" s="2">
         <f>IF(D129=0,"",(H129-D129)/D129)</f>
       </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K129" t="s">
+        <v>64</v>
+      </c>
+      <c r="L129" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="B130">
         <v>24</v>
@@ -4907,10 +5723,16 @@
       <c r="J130" s="2">
         <f>IF(D130=0,"",(H130-D130)/D130)</f>
       </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K130" t="s">
+        <v>64</v>
+      </c>
+      <c r="L130" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="B131">
         <v>266</v>
@@ -4939,10 +5761,16 @@
       <c r="J131" s="2">
         <f>IF(D131=0,"",(H131-D131)/D131)</f>
       </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K131" t="s">
+        <v>64</v>
+      </c>
+      <c r="L131" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="B132">
         <v>270</v>
@@ -4971,10 +5799,16 @@
       <c r="J132" s="2">
         <f>IF(D132=0,"",(H132-D132)/D132)</f>
       </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K132" t="s">
+        <v>64</v>
+      </c>
+      <c r="L132" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="B133">
         <v>296</v>
@@ -5003,10 +5837,16 @@
       <c r="J133" s="2">
         <f>IF(D133=0,"",(H133-D133)/D133)</f>
       </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K133" t="s">
+        <v>64</v>
+      </c>
+      <c r="L133" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="B134">
         <v>75</v>
@@ -5035,16 +5875,22 @@
       <c r="J134" s="2">
         <f>IF(D134=0,"",(H134-D134)/D134)</f>
       </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K134" t="s">
+        <v>26</v>
+      </c>
+      <c r="L134" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="B135">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="C135">
-        <v>1.46</v>
+        <v>1.38</v>
       </c>
       <c r="D135">
         <f>C135*$B$3</f>
@@ -5067,13 +5913,19 @@
       <c r="J135" s="2">
         <f>IF(D135=0,"",(H135-D135)/D135)</f>
       </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K135" t="s">
+        <v>64</v>
+      </c>
+      <c r="L135" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="B136">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C136">
         <v>1.01</v>
@@ -5099,10 +5951,16 @@
       <c r="J136" s="2">
         <f>IF(D136=0,"",(H136-D136)/D136)</f>
       </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K136" t="s">
+        <v>23</v>
+      </c>
+      <c r="L136" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B137">
         <v>310</v>
@@ -5131,13 +5989,19 @@
       <c r="J137" s="2">
         <f>IF(D137=0,"",(H137-D137)/D137)</f>
       </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K137" t="s">
+        <v>23</v>
+      </c>
+      <c r="L137" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="B138">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="C138">
         <v>0.67</v>
@@ -5163,10 +6027,16 @@
       <c r="J138" s="2">
         <f>IF(D138=0,"",(H138-D138)/D138)</f>
       </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K138" t="s">
+        <v>26</v>
+      </c>
+      <c r="L138" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="B139">
         <v>36</v>
@@ -5194,6 +6064,12 @@
       </c>
       <c r="J139" s="2">
         <f>IF(D139=0,"",(H139-D139)/D139)</f>
+      </c>
+      <c r="K139" t="s">
+        <v>58</v>
+      </c>
+      <c r="L139" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>